<commit_message>
Address review: Mermaid extraction, estimate labels, RBAC verification, containment guardrails, Gitleaks
Extract each Mermaid block to its own file before rendering, label sizing assumptions as estimates with a validation plan, add an RBAC console mapping worksheet and verification doc, add ADR-009 with a machine-readable containment policy, and add Gitleaks plus stronger secret-pattern tests.
</commit_message>
<xml_diff>
--- a/01-architecture/sample-data/sizing-calculator.xlsx
+++ b/01-architecture/sample-data/sizing-calculator.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="111">
   <si>
     <t xml:space="preserve">Sizing summary</t>
   </si>
@@ -93,6 +93,9 @@
     <t xml:space="preserve">Depends on compression assumption</t>
   </si>
   <si>
+    <t xml:space="preserve">Basis: all values are ESTIMATES derived from planning inputs (compression 10:1, FortiGate filter 50%, growth 25%). Treat as unvalidated until compared with real telemetry.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Ingest by category (after filtering)</t>
   </si>
   <si>
@@ -141,18 +144,27 @@
     <t xml:space="preserve">Source / note</t>
   </si>
   <si>
+    <t xml:space="preserve">Status</t>
+  </si>
+  <si>
     <t xml:space="preserve">Compression ratio (raw : stored)</t>
   </si>
   <si>
     <t xml:space="preserve">ASSUMPTION - planning value. Measure the real ratio from repository stats after onboarding.</t>
   </si>
   <si>
+    <t xml:space="preserve">ESTIMATE - validate with telemetry</t>
+  </si>
+  <si>
     <t xml:space="preserve">Seconds per day</t>
   </si>
   <si>
     <t xml:space="preserve">Constant.</t>
   </si>
   <si>
+    <t xml:space="preserve">Constant</t>
+  </si>
+  <si>
     <t xml:space="preserve">Bytes per GB (decimal)</t>
   </si>
   <si>
@@ -177,10 +189,19 @@
     <t xml:space="preserve">From author's study notes (Falcon Insight XDR customer). VERIFY against current CrowdStrike licensing.</t>
   </si>
   <si>
+    <t xml:space="preserve">VERIFY against licence</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Per-source EPS, event sizes and pre-ingest filter reductions on the Sizing sheet are also ESTIMATES. Validation plan: docs/03-sizing.md.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Per-source sizing (third-party data only; first-party Falcon data is not counted here)</t>
   </si>
   <si>
     <t xml:space="preserve">LEGEND: edit blue cells (EPS, event size, filter %, retention). Row 5 (Okta) is the example of the expected format. Raw GB/day = EPS x bytes x 86400 / 1e9.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ESTIMATES: EPS, event size and filter reduction (blue cells) are planning values until measured from real telemetry. See docs/03-sizing.md.</t>
   </si>
   <si>
     <t xml:space="preserve">ID</t>
@@ -479,7 +500,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -549,6 +570,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -991,25 +1016,30 @@
         <v>22</v>
       </c>
     </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="9" t="s">
+        <v>23</v>
+      </c>
+    </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="9" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B20" s="10" t="n">
         <f aca="false">SUMIF(Sizing!$C$5:$C$13,A20,Sizing!$J$5:$J$13)</f>
@@ -1022,7 +1052,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B21" s="10" t="n">
         <f aca="false">SUMIF(Sizing!$C$5:$C$13,A21,Sizing!$J$5:$J$13)</f>
@@ -1035,7 +1065,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="3" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B22" s="10" t="n">
         <f aca="false">SUMIF(Sizing!$C$5:$C$13,A22,Sizing!$J$5:$J$13)</f>
@@ -1048,7 +1078,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B23" s="10" t="n">
         <f aca="false">SUMIF(Sizing!$C$5:$C$13,A23,Sizing!$J$5:$J$13)</f>
@@ -1061,7 +1091,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B24" s="10" t="n">
         <f aca="false">SUMIF(Sizing!$C$5:$C$13,A24,Sizing!$J$5:$J$13)</f>
@@ -1074,7 +1104,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="3" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B25" s="10" t="n">
         <f aca="false">SUMIF(Sizing!$C$5:$C$13,A25,Sizing!$J$5:$J$13)</f>
@@ -1087,7 +1117,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="9" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B26" s="12" t="n">
         <f aca="false">SUM(B20:B25)</f>
@@ -1100,7 +1130,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="14" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B27" s="14" t="str">
         <f aca="false">IF(ABS(B26-B9)&lt;0.0001,"OK","MISMATCH")</f>
@@ -1123,101 +1153,128 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="38"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="85"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="34"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="15" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B2" s="15"/>
       <c r="C2" s="15"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>2</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B5" s="16" t="n">
         <v>10</v>
       </c>
       <c r="C5" s="17" t="s">
-        <v>40</v>
+        <v>42</v>
+      </c>
+      <c r="D5" s="18" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="B6" s="18" t="n">
+        <v>44</v>
+      </c>
+      <c r="B6" s="19" t="n">
         <v>86400</v>
       </c>
       <c r="C6" s="17" t="s">
-        <v>42</v>
+        <v>45</v>
+      </c>
+      <c r="D6" s="17" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="B7" s="18" t="n">
+        <v>47</v>
+      </c>
+      <c r="B7" s="19" t="n">
         <v>1000000000</v>
       </c>
       <c r="C7" s="17" t="s">
-        <v>44</v>
+        <v>48</v>
+      </c>
+      <c r="D7" s="17" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="B8" s="19" t="n">
+        <v>49</v>
+      </c>
+      <c r="B8" s="20" t="n">
         <v>0.25</v>
       </c>
       <c r="C8" s="17" t="s">
-        <v>46</v>
+        <v>50</v>
+      </c>
+      <c r="D8" s="18" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="B9" s="16" t="n">
         <v>3</v>
       </c>
       <c r="C9" s="17" t="s">
-        <v>48</v>
+        <v>52</v>
+      </c>
+      <c r="D9" s="18" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="B10" s="20" t="n">
+        <v>53</v>
+      </c>
+      <c r="B10" s="21" t="n">
         <v>10</v>
       </c>
       <c r="C10" s="17" t="s">
-        <v>50</v>
+        <v>54</v>
+      </c>
+      <c r="D10" s="18" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="9" t="s">
+        <v>56</v>
       </c>
     </row>
   </sheetData>
@@ -1258,89 +1315,94 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="14" t="s">
-        <v>52</v>
+        <v>58</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="9" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>53</v>
+        <v>60</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>58</v>
+        <v>65</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>61</v>
+        <v>68</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="M4" s="2" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="17" t="s">
-        <v>64</v>
+        <v>71</v>
       </c>
       <c r="B5" s="17" t="s">
-        <v>65</v>
+        <v>72</v>
       </c>
       <c r="C5" s="17" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D5" s="17" t="s">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="E5" s="17" t="s">
-        <v>67</v>
-      </c>
-      <c r="F5" s="18" t="n">
+        <v>74</v>
+      </c>
+      <c r="F5" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="G5" s="18" t="n">
+      <c r="G5" s="19" t="n">
         <v>900</v>
       </c>
       <c r="H5" s="10" t="n">
         <f aca="false">F5*G5*Assumptions!$B$6/Assumptions!$B$7</f>
         <v>0.23328</v>
       </c>
-      <c r="I5" s="21" t="n">
+      <c r="I5" s="22" t="n">
         <v>0</v>
       </c>
       <c r="J5" s="10" t="n">
         <f aca="false">H5*(1-I5)</f>
         <v>0.23328</v>
       </c>
-      <c r="K5" s="18" t="n">
+      <c r="K5" s="19" t="n">
         <v>365</v>
       </c>
       <c r="L5" s="8" t="n">
@@ -1348,43 +1410,43 @@
         <v>8.51472</v>
       </c>
       <c r="M5" s="17" t="s">
-        <v>68</v>
+        <v>75</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="17" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="B6" s="17" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="C6" s="17" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D6" s="17" t="s">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="E6" s="17" t="s">
-        <v>67</v>
-      </c>
-      <c r="F6" s="18" t="n">
+        <v>74</v>
+      </c>
+      <c r="F6" s="19" t="n">
         <v>4</v>
       </c>
-      <c r="G6" s="18" t="n">
+      <c r="G6" s="19" t="n">
         <v>1200</v>
       </c>
       <c r="H6" s="10" t="n">
         <f aca="false">F6*G6*Assumptions!$B$6/Assumptions!$B$7</f>
         <v>0.41472</v>
       </c>
-      <c r="I6" s="21" t="n">
+      <c r="I6" s="22" t="n">
         <v>0</v>
       </c>
       <c r="J6" s="10" t="n">
         <f aca="false">H6*(1-I6)</f>
         <v>0.41472</v>
       </c>
-      <c r="K6" s="18" t="n">
+      <c r="K6" s="19" t="n">
         <v>365</v>
       </c>
       <c r="L6" s="8" t="n">
@@ -1392,43 +1454,43 @@
         <v>15.13728</v>
       </c>
       <c r="M6" s="17" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="17" t="s">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="B7" s="17" t="s">
+        <v>80</v>
+      </c>
+      <c r="C7" s="17" t="s">
+        <v>29</v>
+      </c>
+      <c r="D7" s="17" t="s">
         <v>73</v>
       </c>
-      <c r="C7" s="17" t="s">
-        <v>28</v>
-      </c>
-      <c r="D7" s="17" t="s">
-        <v>66</v>
-      </c>
       <c r="E7" s="17" t="s">
-        <v>74</v>
-      </c>
-      <c r="F7" s="18" t="n">
+        <v>81</v>
+      </c>
+      <c r="F7" s="19" t="n">
         <v>6</v>
       </c>
-      <c r="G7" s="18" t="n">
+      <c r="G7" s="19" t="n">
         <v>1000</v>
       </c>
       <c r="H7" s="10" t="n">
         <f aca="false">F7*G7*Assumptions!$B$6/Assumptions!$B$7</f>
         <v>0.5184</v>
       </c>
-      <c r="I7" s="21" t="n">
+      <c r="I7" s="22" t="n">
         <v>0</v>
       </c>
       <c r="J7" s="10" t="n">
         <f aca="false">H7*(1-I7)</f>
         <v>0.5184</v>
       </c>
-      <c r="K7" s="18" t="n">
+      <c r="K7" s="19" t="n">
         <v>365</v>
       </c>
       <c r="L7" s="8" t="n">
@@ -1436,43 +1498,43 @@
         <v>18.9216</v>
       </c>
       <c r="M7" s="17" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="17" t="s">
-        <v>76</v>
+        <v>83</v>
       </c>
       <c r="B8" s="17" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="C8" s="17" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D8" s="17" t="s">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="E8" s="17" t="s">
-        <v>78</v>
-      </c>
-      <c r="F8" s="18" t="n">
+        <v>85</v>
+      </c>
+      <c r="F8" s="19" t="n">
         <v>8</v>
       </c>
-      <c r="G8" s="18" t="n">
+      <c r="G8" s="19" t="n">
         <v>1100</v>
       </c>
       <c r="H8" s="10" t="n">
         <f aca="false">F8*G8*Assumptions!$B$6/Assumptions!$B$7</f>
         <v>0.76032</v>
       </c>
-      <c r="I8" s="21" t="n">
+      <c r="I8" s="22" t="n">
         <v>0</v>
       </c>
       <c r="J8" s="10" t="n">
         <f aca="false">H8*(1-I8)</f>
         <v>0.76032</v>
       </c>
-      <c r="K8" s="18" t="n">
+      <c r="K8" s="19" t="n">
         <v>365</v>
       </c>
       <c r="L8" s="8" t="n">
@@ -1480,43 +1542,43 @@
         <v>27.75168</v>
       </c>
       <c r="M8" s="17" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="17" t="s">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="B9" s="17" t="s">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="C9" s="17" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D9" s="17" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="E9" s="17" t="s">
-        <v>83</v>
-      </c>
-      <c r="F9" s="18" t="n">
+        <v>90</v>
+      </c>
+      <c r="F9" s="19" t="n">
         <v>100</v>
       </c>
-      <c r="G9" s="18" t="n">
+      <c r="G9" s="19" t="n">
         <v>550</v>
       </c>
       <c r="H9" s="10" t="n">
         <f aca="false">F9*G9*Assumptions!$B$6/Assumptions!$B$7</f>
         <v>4.752</v>
       </c>
-      <c r="I9" s="21" t="n">
+      <c r="I9" s="22" t="n">
         <v>0.5</v>
       </c>
       <c r="J9" s="10" t="n">
         <f aca="false">H9*(1-I9)</f>
         <v>2.376</v>
       </c>
-      <c r="K9" s="18" t="n">
+      <c r="K9" s="19" t="n">
         <v>90</v>
       </c>
       <c r="L9" s="8" t="n">
@@ -1524,43 +1586,43 @@
         <v>21.384</v>
       </c>
       <c r="M9" s="17" t="s">
-        <v>84</v>
+        <v>91</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="17" t="s">
-        <v>85</v>
+        <v>92</v>
       </c>
       <c r="B10" s="17" t="s">
-        <v>86</v>
+        <v>93</v>
       </c>
       <c r="C10" s="17" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D10" s="17" t="s">
-        <v>87</v>
+        <v>94</v>
       </c>
       <c r="E10" s="17" t="s">
-        <v>88</v>
-      </c>
-      <c r="F10" s="18" t="n">
+        <v>95</v>
+      </c>
+      <c r="F10" s="19" t="n">
         <v>8</v>
       </c>
-      <c r="G10" s="18" t="n">
+      <c r="G10" s="19" t="n">
         <v>700</v>
       </c>
       <c r="H10" s="10" t="n">
         <f aca="false">F10*G10*Assumptions!$B$6/Assumptions!$B$7</f>
         <v>0.48384</v>
       </c>
-      <c r="I10" s="21" t="n">
+      <c r="I10" s="22" t="n">
         <v>0</v>
       </c>
       <c r="J10" s="10" t="n">
         <f aca="false">H10*(1-I10)</f>
         <v>0.48384</v>
       </c>
-      <c r="K10" s="18" t="n">
+      <c r="K10" s="19" t="n">
         <v>180</v>
       </c>
       <c r="L10" s="8" t="n">
@@ -1568,43 +1630,43 @@
         <v>8.70912</v>
       </c>
       <c r="M10" s="17" t="s">
-        <v>89</v>
+        <v>96</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="17" t="s">
+        <v>97</v>
+      </c>
+      <c r="B11" s="17" t="s">
+        <v>98</v>
+      </c>
+      <c r="C11" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="D11" s="17" t="s">
+        <v>99</v>
+      </c>
+      <c r="E11" s="17" t="s">
         <v>90</v>
       </c>
-      <c r="B11" s="17" t="s">
-        <v>91</v>
-      </c>
-      <c r="C11" s="17" t="s">
-        <v>31</v>
-      </c>
-      <c r="D11" s="17" t="s">
-        <v>92</v>
-      </c>
-      <c r="E11" s="17" t="s">
-        <v>83</v>
-      </c>
-      <c r="F11" s="18" t="n">
+      <c r="F11" s="19" t="n">
         <v>40</v>
       </c>
-      <c r="G11" s="18" t="n">
+      <c r="G11" s="19" t="n">
         <v>700</v>
       </c>
       <c r="H11" s="10" t="n">
         <f aca="false">F11*G11*Assumptions!$B$6/Assumptions!$B$7</f>
         <v>2.4192</v>
       </c>
-      <c r="I11" s="21" t="n">
+      <c r="I11" s="22" t="n">
         <v>0.25</v>
       </c>
       <c r="J11" s="10" t="n">
         <f aca="false">H11*(1-I11)</f>
         <v>1.8144</v>
       </c>
-      <c r="K11" s="18" t="n">
+      <c r="K11" s="19" t="n">
         <v>90</v>
       </c>
       <c r="L11" s="8" t="n">
@@ -1612,43 +1674,43 @@
         <v>16.3296</v>
       </c>
       <c r="M11" s="17" t="s">
-        <v>93</v>
+        <v>100</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="17" t="s">
-        <v>94</v>
+        <v>101</v>
       </c>
       <c r="B12" s="17" t="s">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="C12" s="17" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D12" s="17" t="s">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="E12" s="17" t="s">
-        <v>97</v>
-      </c>
-      <c r="F12" s="18" t="n">
+        <v>104</v>
+      </c>
+      <c r="F12" s="19" t="n">
         <v>25</v>
       </c>
-      <c r="G12" s="18" t="n">
+      <c r="G12" s="19" t="n">
         <v>800</v>
       </c>
       <c r="H12" s="10" t="n">
         <f aca="false">F12*G12*Assumptions!$B$6/Assumptions!$B$7</f>
         <v>1.728</v>
       </c>
-      <c r="I12" s="21" t="n">
+      <c r="I12" s="22" t="n">
         <v>0.3</v>
       </c>
       <c r="J12" s="10" t="n">
         <f aca="false">H12*(1-I12)</f>
         <v>1.2096</v>
       </c>
-      <c r="K12" s="18" t="n">
+      <c r="K12" s="19" t="n">
         <v>180</v>
       </c>
       <c r="L12" s="8" t="n">
@@ -1656,43 +1718,43 @@
         <v>21.7728</v>
       </c>
       <c r="M12" s="17" t="s">
-        <v>98</v>
+        <v>105</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="17" t="s">
-        <v>99</v>
+        <v>106</v>
       </c>
       <c r="B13" s="17" t="s">
-        <v>100</v>
+        <v>107</v>
       </c>
       <c r="C13" s="17" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D13" s="17" t="s">
-        <v>101</v>
+        <v>108</v>
       </c>
       <c r="E13" s="17" t="s">
-        <v>97</v>
-      </c>
-      <c r="F13" s="18" t="n">
+        <v>104</v>
+      </c>
+      <c r="F13" s="19" t="n">
         <v>10</v>
       </c>
-      <c r="G13" s="18" t="n">
+      <c r="G13" s="19" t="n">
         <v>250</v>
       </c>
       <c r="H13" s="10" t="n">
         <f aca="false">F13*G13*Assumptions!$B$6/Assumptions!$B$7</f>
         <v>0.216</v>
       </c>
-      <c r="I13" s="21" t="n">
+      <c r="I13" s="22" t="n">
         <v>0</v>
       </c>
       <c r="J13" s="10" t="n">
         <f aca="false">H13*(1-I13)</f>
         <v>0.216</v>
       </c>
-      <c r="K13" s="18" t="n">
+      <c r="K13" s="19" t="n">
         <v>180</v>
       </c>
       <c r="L13" s="8" t="n">
@@ -1700,33 +1762,33 @@
         <v>3.888</v>
       </c>
       <c r="M13" s="17" t="s">
-        <v>102</v>
+        <v>109</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="9" t="s">
-        <v>33</v>
-      </c>
-      <c r="F14" s="22" t="n">
+        <v>34</v>
+      </c>
+      <c r="F14" s="23" t="n">
         <f aca="false">SUM(F5:F13)</f>
         <v>204</v>
       </c>
-      <c r="H14" s="23" t="n">
+      <c r="H14" s="24" t="n">
         <f aca="false">SUM(H5:H13)</f>
         <v>11.52576</v>
       </c>
-      <c r="J14" s="23" t="n">
+      <c r="J14" s="24" t="n">
         <f aca="false">SUM(J5:J13)</f>
         <v>8.02656</v>
       </c>
-      <c r="L14" s="24" t="n">
+      <c r="L14" s="25" t="n">
         <f aca="false">SUM(L5:L13)</f>
         <v>142.4088</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="14" t="s">
-        <v>103</v>
+        <v>110</v>
       </c>
     </row>
   </sheetData>

</xml_diff>